<commit_message>
feat: Add core utilities, workflow module, and tutorials, and enhance `uhi_morph` function with improved error handling.
</commit_message>
<xml_diff>
--- a/docs/source/tutorials/my_parametric_study.xlsx
+++ b/docs/source/tutorials/my_parametric_study.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>epw_paths</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t>fwg_target_uhi_lcz</t>
+  </si>
+  <si>
+    <t>fwg_output_type</t>
+  </si>
+  <si>
+    <t>fwg_version</t>
   </si>
 </sst>
 </file>
@@ -446,10 +452,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:27">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -524,6 +530,12 @@
       </c>
       <c r="Y1" s="1" t="s">
         <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>